<commit_message>
Resolved Failed Test cases- 11-Jun-2026
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/Modules/09_MyWebSite/MyWebSite/02_WebSite_Resubmit.xlsx
+++ b/src/test/resources/testdata/Modules/09_MyWebSite/MyWebSite/02_WebSite_Resubmit.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\testing\Documents\Bandhan_World_APPIUM\src\test\resources\testdata\Modules\09_MyWebSite\MyWebSite\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{756DFDFE-872F-4CCD-B836-345BEE4519C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{022BA03F-DDCC-4736-95E6-4ED350673D5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="1" xr2:uid="{D5674106-8292-4F40-9DFC-E6EAC771FC2F}"/>
   </bookViews>
@@ -1212,13 +1212,6 @@
 verify_iswebsite_created</t>
   </si>
   <si>
-    <t>approve_website
-relaunchappwithoutdataclear
-clickonskipbtnofinsurancewindow
-open_mywebsitemenu
-verify_mywebsite_webversion_status</t>
-  </si>
-  <si>
     <t>Rejected And Pending For Resubmission</t>
   </si>
   <si>
@@ -1678,6 +1671,13 @@
 open_mywebsitemenu
 clickon_website_fabbtn
 verify_editsite_website_status</t>
+  </si>
+  <si>
+    <t>approve_website
+relaunchappwithoutdataclear
+clickonskipbtnofinsurancewindow
+open_mywebsitemenu
+verify_resubmit_webvesrion_status</t>
   </si>
 </sst>
 </file>
@@ -2717,7 +2717,7 @@
         <v>75</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>204</v>
+        <v>311</v>
       </c>
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
@@ -2727,7 +2727,7 @@
       <c r="K3" s="3"/>
       <c r="L3" s="3"/>
       <c r="M3" s="3" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="N3" s="3" t="s">
         <v>5</v>
@@ -2741,13 +2741,13 @@
         <v>11</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>74</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="F4" s="3"/>
       <c r="G4" s="3"/>
@@ -2757,7 +2757,7 @@
       <c r="K4" s="3"/>
       <c r="L4" s="3"/>
       <c r="M4" s="3" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="N4" s="3" t="s">
         <v>5</v>
@@ -2777,7 +2777,7 @@
         <v>77</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="F5" s="3"/>
       <c r="G5" s="3"/>
@@ -2787,7 +2787,7 @@
       <c r="K5" s="3"/>
       <c r="L5" s="3"/>
       <c r="M5" s="3" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="N5" s="3" t="s">
         <v>5</v>
@@ -2807,7 +2807,7 @@
         <v>78</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F6" s="3"/>
       <c r="G6" s="3"/>
@@ -2817,7 +2817,7 @@
       <c r="K6" s="3"/>
       <c r="L6" s="3"/>
       <c r="M6" s="3" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N6" s="3" t="s">
         <v>5</v>
@@ -2837,7 +2837,7 @@
         <v>79</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="F7" s="3"/>
       <c r="G7" s="3"/>
@@ -2867,7 +2867,7 @@
         <v>80</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="F8" s="3"/>
       <c r="G8" s="3"/>
@@ -2877,7 +2877,7 @@
       <c r="K8" s="3"/>
       <c r="L8" s="3"/>
       <c r="M8" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="N8" s="3" t="s">
         <v>5</v>
@@ -2897,7 +2897,7 @@
         <v>81</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="F9" s="3"/>
       <c r="G9" s="3"/>
@@ -2907,7 +2907,7 @@
       <c r="K9" s="3"/>
       <c r="L9" s="3"/>
       <c r="M9" s="8" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="N9" s="3" t="s">
         <v>5</v>
@@ -2927,7 +2927,7 @@
         <v>82</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="F10" s="3"/>
       <c r="G10" s="3"/>
@@ -2937,7 +2937,7 @@
       <c r="K10" s="3"/>
       <c r="L10" s="3"/>
       <c r="M10" s="8" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="N10" s="3" t="s">
         <v>5</v>
@@ -2957,7 +2957,7 @@
         <v>83</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="F11" s="3"/>
       <c r="G11" s="3"/>
@@ -2967,7 +2967,7 @@
       <c r="K11" s="3"/>
       <c r="L11" s="3"/>
       <c r="M11" s="8" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="N11" s="3" t="s">
         <v>5</v>
@@ -2987,7 +2987,7 @@
         <v>84</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="F12" s="3"/>
       <c r="G12" s="3"/>
@@ -2997,7 +2997,7 @@
       <c r="K12" s="3"/>
       <c r="L12" s="3"/>
       <c r="M12" s="8" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="N12" s="3" t="s">
         <v>5</v>
@@ -3014,10 +3014,10 @@
         <v>138</v>
       </c>
       <c r="D13" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="E13" s="3" t="s">
         <v>216</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>217</v>
       </c>
       <c r="F13" s="3"/>
       <c r="G13" s="3"/>
@@ -3027,7 +3027,7 @@
       <c r="K13" s="3"/>
       <c r="L13" s="3"/>
       <c r="M13" s="8" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="N13" s="3" t="s">
         <v>5</v>
@@ -3047,7 +3047,7 @@
         <v>85</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="F14" s="3"/>
       <c r="G14" s="3"/>
@@ -3057,7 +3057,7 @@
       <c r="K14" s="3"/>
       <c r="L14" s="3"/>
       <c r="M14" s="8" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="N14" s="3" t="s">
         <v>5</v>
@@ -3077,10 +3077,10 @@
         <v>86</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="G15" s="3"/>
       <c r="H15" s="3"/>
@@ -3089,7 +3089,7 @@
       <c r="K15" s="3"/>
       <c r="L15" s="3"/>
       <c r="M15" s="3" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="N15" s="3" t="s">
         <v>5</v>
@@ -3109,7 +3109,7 @@
         <v>87</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="F16" s="3"/>
       <c r="G16" s="3"/>
@@ -3119,7 +3119,7 @@
       <c r="K16" s="3"/>
       <c r="L16" s="3"/>
       <c r="M16" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="N16" s="3" t="s">
         <v>5</v>
@@ -3139,10 +3139,10 @@
         <v>88</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="G17" s="3"/>
       <c r="H17" s="3"/>
@@ -3171,7 +3171,7 @@
         <v>89</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="F18" s="3"/>
       <c r="G18" s="3"/>
@@ -3181,7 +3181,7 @@
       <c r="K18" s="3"/>
       <c r="L18" s="3"/>
       <c r="M18" s="3" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="N18" s="3" t="s">
         <v>5</v>
@@ -3201,7 +3201,7 @@
         <v>90</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="F19" s="3"/>
       <c r="G19" s="3"/>
@@ -3211,7 +3211,7 @@
       <c r="K19" s="3"/>
       <c r="L19" s="3"/>
       <c r="M19" s="3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="N19" s="3" t="s">
         <v>5</v>
@@ -3231,7 +3231,7 @@
         <v>91</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="F20" s="3"/>
       <c r="G20" s="3"/>
@@ -3241,7 +3241,7 @@
       <c r="K20" s="3"/>
       <c r="L20" s="3"/>
       <c r="M20" s="3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="N20" s="3" t="s">
         <v>5</v>
@@ -3261,7 +3261,7 @@
         <v>92</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="F21" s="3"/>
       <c r="G21" s="3"/>
@@ -3271,7 +3271,7 @@
       <c r="K21" s="3"/>
       <c r="L21" s="3"/>
       <c r="M21" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="N21" s="3" t="s">
         <v>5</v>
@@ -3291,7 +3291,7 @@
         <v>93</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="F22" s="3"/>
       <c r="G22" s="3"/>
@@ -3321,7 +3321,7 @@
         <v>94</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="F23" s="3"/>
       <c r="G23" s="3"/>
@@ -3331,7 +3331,7 @@
       <c r="K23" s="3"/>
       <c r="L23" s="3"/>
       <c r="M23" s="8" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="N23" s="3" t="s">
         <v>5</v>
@@ -3351,7 +3351,7 @@
         <v>95</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="F24" s="3"/>
       <c r="G24" s="3"/>
@@ -3361,7 +3361,7 @@
       <c r="K24" s="3"/>
       <c r="L24" s="3"/>
       <c r="M24" s="8" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="N24" s="3" t="s">
         <v>5</v>
@@ -3375,13 +3375,13 @@
         <v>11</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="D25" s="3" t="s">
         <v>96</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="F25" s="3"/>
       <c r="G25" s="3"/>
@@ -3391,7 +3391,7 @@
       <c r="K25" s="3"/>
       <c r="L25" s="3"/>
       <c r="M25" s="8" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="N25" s="3" t="s">
         <v>5</v>
@@ -3411,7 +3411,7 @@
         <v>97</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="F26" s="3"/>
       <c r="G26" s="3"/>
@@ -3421,7 +3421,7 @@
       <c r="K26" s="3"/>
       <c r="L26" s="3"/>
       <c r="M26" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="N26" s="3" t="s">
         <v>5</v>
@@ -3441,7 +3441,7 @@
         <v>98</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="F27" s="3"/>
       <c r="G27" s="3"/>
@@ -3471,7 +3471,7 @@
         <v>99</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="F28" s="3"/>
       <c r="G28" s="3"/>
@@ -3481,7 +3481,7 @@
       <c r="K28" s="3"/>
       <c r="L28" s="3"/>
       <c r="M28" s="8" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="N28" s="3" t="s">
         <v>5</v>
@@ -3501,7 +3501,7 @@
         <v>100</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="F29" s="3"/>
       <c r="G29" s="3"/>
@@ -3511,7 +3511,7 @@
       <c r="K29" s="3"/>
       <c r="L29" s="3"/>
       <c r="M29" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="N29" s="3" t="s">
         <v>5</v>
@@ -3531,10 +3531,10 @@
         <v>101</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="G30" s="3"/>
       <c r="H30" s="3"/>
@@ -3563,7 +3563,7 @@
         <v>102</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="F31" s="3"/>
       <c r="G31" s="3"/>
@@ -3573,7 +3573,7 @@
       <c r="K31" s="3"/>
       <c r="L31" s="3"/>
       <c r="M31" s="4" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="N31" s="3" t="s">
         <v>5</v>
@@ -3590,10 +3590,10 @@
         <v>156</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="F32" s="3"/>
       <c r="G32" s="3"/>
@@ -3603,7 +3603,7 @@
       <c r="K32" s="3"/>
       <c r="L32" s="3"/>
       <c r="M32" s="3" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="N32" s="3" t="s">
         <v>5</v>
@@ -3620,10 +3620,10 @@
         <v>157</v>
       </c>
       <c r="D33" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="E33" s="3" t="s">
         <v>244</v>
-      </c>
-      <c r="E33" s="3" t="s">
-        <v>245</v>
       </c>
       <c r="F33" s="3"/>
       <c r="G33" s="3"/>
@@ -3653,7 +3653,7 @@
         <v>103</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="F34" s="3"/>
       <c r="G34" s="3"/>
@@ -3677,13 +3677,13 @@
         <v>11</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="F35" s="3"/>
       <c r="G35" s="3"/>
@@ -3693,7 +3693,7 @@
       <c r="K35" s="3"/>
       <c r="L35" s="3"/>
       <c r="M35" s="8" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="N35" s="3" t="s">
         <v>5</v>
@@ -3710,10 +3710,10 @@
         <v>159</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F36" s="3"/>
       <c r="G36" s="3"/>
@@ -3723,7 +3723,7 @@
       <c r="K36" s="3"/>
       <c r="L36" s="3"/>
       <c r="M36" s="8" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="N36" s="3" t="s">
         <v>5</v>
@@ -3740,10 +3740,10 @@
         <v>160</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="F37" s="3"/>
       <c r="G37" s="3"/>
@@ -3753,7 +3753,7 @@
       <c r="K37" s="3"/>
       <c r="L37" s="3"/>
       <c r="M37" s="8" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="N37" s="3" t="s">
         <v>5</v>
@@ -3773,7 +3773,7 @@
         <v>104</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="F38" s="3"/>
       <c r="G38" s="3"/>
@@ -3783,7 +3783,7 @@
       <c r="K38" s="3"/>
       <c r="L38" s="3"/>
       <c r="M38" s="8" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="N38" s="3" t="s">
         <v>5</v>
@@ -3803,7 +3803,7 @@
         <v>105</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="F39" s="3"/>
       <c r="G39" s="3"/>
@@ -3813,7 +3813,7 @@
       <c r="K39" s="3"/>
       <c r="L39" s="3"/>
       <c r="M39" s="8" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="N39" s="3" t="s">
         <v>5</v>
@@ -3833,7 +3833,7 @@
         <v>106</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="F40" s="3"/>
       <c r="G40" s="3"/>
@@ -3843,7 +3843,7 @@
       <c r="K40" s="3"/>
       <c r="L40" s="3"/>
       <c r="M40" s="8" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="N40" s="3" t="s">
         <v>5</v>
@@ -3863,7 +3863,7 @@
         <v>107</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="F41" s="3"/>
       <c r="G41" s="3"/>
@@ -3873,7 +3873,7 @@
       <c r="K41" s="3"/>
       <c r="L41" s="3"/>
       <c r="M41" s="8" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="N41" s="3" t="s">
         <v>5</v>
@@ -3893,7 +3893,7 @@
         <v>108</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="F42" s="3"/>
       <c r="G42" s="3"/>
@@ -3923,7 +3923,7 @@
         <v>109</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="F43" s="3"/>
       <c r="G43" s="3"/>
@@ -3953,7 +3953,7 @@
         <v>110</v>
       </c>
       <c r="E44" s="3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="F44" s="3"/>
       <c r="G44" s="3"/>
@@ -3963,7 +3963,7 @@
       <c r="K44" s="3"/>
       <c r="L44" s="3"/>
       <c r="M44" s="8" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="N44" s="3" t="s">
         <v>5</v>
@@ -3983,7 +3983,7 @@
         <v>111</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="F45" s="3"/>
       <c r="G45" s="3"/>
@@ -3993,7 +3993,7 @@
       <c r="K45" s="3"/>
       <c r="L45" s="3"/>
       <c r="M45" s="8" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="N45" s="3" t="s">
         <v>5</v>
@@ -4013,21 +4013,21 @@
         <v>112</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F46" s="3" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="G46" s="3"/>
       <c r="H46" s="9" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="I46" s="3"/>
       <c r="J46" s="3"/>
       <c r="K46" s="3"/>
       <c r="L46" s="3"/>
       <c r="M46" s="3" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="N46" s="3" t="s">
         <v>5</v>
@@ -4047,7 +4047,7 @@
         <v>113</v>
       </c>
       <c r="E47" s="3" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F47" s="3"/>
       <c r="G47" s="3"/>
@@ -4057,7 +4057,7 @@
       <c r="K47" s="3"/>
       <c r="L47" s="3"/>
       <c r="M47" s="3" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="N47" s="3" t="s">
         <v>5</v>
@@ -4077,7 +4077,7 @@
         <v>114</v>
       </c>
       <c r="E48" s="3" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="F48" s="3"/>
       <c r="G48" s="3"/>
@@ -4087,7 +4087,7 @@
       <c r="K48" s="3"/>
       <c r="L48" s="3"/>
       <c r="M48" s="8" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="N48" s="3" t="s">
         <v>5</v>
@@ -4107,7 +4107,7 @@
         <v>115</v>
       </c>
       <c r="E49" s="3" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="F49" s="3"/>
       <c r="G49" s="3"/>
@@ -4117,7 +4117,7 @@
       <c r="K49" s="3"/>
       <c r="L49" s="3"/>
       <c r="M49" s="8" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="N49" s="3" t="s">
         <v>5</v>
@@ -4137,7 +4137,7 @@
         <v>116</v>
       </c>
       <c r="E50" s="3" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="F50" s="3"/>
       <c r="G50" s="3"/>
@@ -4167,7 +4167,7 @@
         <v>117</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="F51" s="3"/>
       <c r="G51" s="3"/>
@@ -4177,7 +4177,7 @@
       <c r="K51" s="3"/>
       <c r="L51" s="3"/>
       <c r="M51" s="3" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="N51" s="3" t="s">
         <v>5</v>
@@ -4197,21 +4197,21 @@
         <v>118</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F52" s="3" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="G52" s="3"/>
       <c r="H52" s="9" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="I52" s="3"/>
       <c r="J52" s="3"/>
       <c r="K52" s="3"/>
       <c r="L52" s="3"/>
       <c r="M52" s="8" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="N52" s="3" t="s">
         <v>5</v>
@@ -4231,7 +4231,7 @@
         <v>119</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="F53" s="3"/>
       <c r="G53" s="3"/>
@@ -4241,7 +4241,7 @@
       <c r="K53" s="3"/>
       <c r="L53" s="3"/>
       <c r="M53" s="3" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="N53" s="3" t="s">
         <v>5</v>
@@ -4261,7 +4261,7 @@
         <v>120</v>
       </c>
       <c r="E54" s="3" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="F54" s="3"/>
       <c r="G54" s="3"/>
@@ -4271,7 +4271,7 @@
       <c r="K54" s="3"/>
       <c r="L54" s="3"/>
       <c r="M54" s="8" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="N54" s="3" t="s">
         <v>5</v>
@@ -4291,7 +4291,7 @@
         <v>121</v>
       </c>
       <c r="E55" s="3" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="F55" s="3"/>
       <c r="G55" s="3"/>
@@ -4321,7 +4321,7 @@
         <v>122</v>
       </c>
       <c r="E56" s="3" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="F56" s="3"/>
       <c r="G56" s="3"/>
@@ -4331,7 +4331,7 @@
       <c r="K56" s="3"/>
       <c r="L56" s="3"/>
       <c r="M56" s="8" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="N56" s="3" t="s">
         <v>5</v>
@@ -4351,7 +4351,7 @@
         <v>123</v>
       </c>
       <c r="E57" s="3" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="F57" s="3"/>
       <c r="G57" s="3"/>
@@ -4361,7 +4361,7 @@
       <c r="K57" s="3"/>
       <c r="L57" s="3"/>
       <c r="M57" s="8" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="N57" s="3" t="s">
         <v>5</v>
@@ -4693,7 +4693,7 @@
         <v>22</v>
       </c>
       <c r="E68" s="3" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="F68" s="3"/>
       <c r="G68" s="3"/>
@@ -4729,7 +4729,7 @@
         <v>124</v>
       </c>
       <c r="E69" s="3" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="F69" s="3"/>
       <c r="G69" s="3"/>
@@ -4739,7 +4739,7 @@
       <c r="K69" s="3"/>
       <c r="L69" s="3"/>
       <c r="M69" s="8" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="N69" s="3" t="s">
         <v>5</v>
@@ -4759,7 +4759,7 @@
         <v>125</v>
       </c>
       <c r="E70" s="3" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="F70" s="3"/>
       <c r="G70" s="3"/>
@@ -4787,7 +4787,7 @@
         <v>126</v>
       </c>
       <c r="E71" s="3" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="F71" s="3"/>
       <c r="G71" s="3"/>
@@ -4797,7 +4797,7 @@
       <c r="K71" s="3"/>
       <c r="L71" s="3"/>
       <c r="M71" s="6" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="N71" s="3" t="s">
         <v>5</v>
@@ -4857,7 +4857,7 @@
       <c r="K73" s="3"/>
       <c r="L73" s="3"/>
       <c r="M73" s="6" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="N73" s="3" t="s">
         <v>5</v>
@@ -4997,7 +4997,7 @@
         <v>29</v>
       </c>
       <c r="E78" s="3" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F78" s="3"/>
       <c r="G78" s="3"/>
@@ -5027,7 +5027,7 @@
         <v>127</v>
       </c>
       <c r="E79" s="3" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="F79" s="3"/>
       <c r="G79" s="3"/>
@@ -5037,7 +5037,7 @@
       <c r="K79" s="3"/>
       <c r="L79" s="3"/>
       <c r="M79" s="6" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="N79" s="3" t="s">
         <v>5</v>
@@ -5160,7 +5160,7 @@
         <v>75</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>204</v>
+        <v>311</v>
       </c>
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
@@ -5170,7 +5170,7 @@
       <c r="K3" s="3"/>
       <c r="L3" s="3"/>
       <c r="M3" s="3" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="N3" s="3" t="s">
         <v>5</v>
@@ -5184,13 +5184,13 @@
         <v>11</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>74</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="F4" s="3"/>
       <c r="G4" s="3"/>
@@ -5200,7 +5200,7 @@
       <c r="K4" s="3"/>
       <c r="L4" s="3"/>
       <c r="M4" s="3" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="N4" s="3" t="s">
         <v>5</v>
@@ -5220,7 +5220,7 @@
         <v>77</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="F5" s="3"/>
       <c r="G5" s="3"/>
@@ -5230,7 +5230,7 @@
       <c r="K5" s="3"/>
       <c r="L5" s="3"/>
       <c r="M5" s="3" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="N5" s="3" t="s">
         <v>5</v>
@@ -5250,7 +5250,7 @@
         <v>78</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F6" s="3"/>
       <c r="G6" s="3"/>
@@ -5260,7 +5260,7 @@
       <c r="K6" s="3"/>
       <c r="L6" s="3"/>
       <c r="M6" s="3" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N6" s="3" t="s">
         <v>5</v>
@@ -5280,7 +5280,7 @@
         <v>79</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="F7" s="3"/>
       <c r="G7" s="3"/>
@@ -5310,7 +5310,7 @@
         <v>80</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="F8" s="3"/>
       <c r="G8" s="3"/>
@@ -5320,7 +5320,7 @@
       <c r="K8" s="3"/>
       <c r="L8" s="3"/>
       <c r="M8" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="N8" s="3" t="s">
         <v>5</v>
@@ -5340,7 +5340,7 @@
         <v>81</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="F9" s="3"/>
       <c r="G9" s="3"/>
@@ -5350,7 +5350,7 @@
       <c r="K9" s="3"/>
       <c r="L9" s="3"/>
       <c r="M9" s="8" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="N9" s="3" t="s">
         <v>5</v>
@@ -5370,7 +5370,7 @@
         <v>82</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="F10" s="3"/>
       <c r="G10" s="3"/>
@@ -5380,7 +5380,7 @@
       <c r="K10" s="3"/>
       <c r="L10" s="3"/>
       <c r="M10" s="8" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="N10" s="3" t="s">
         <v>5</v>
@@ -5400,7 +5400,7 @@
         <v>83</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="F11" s="3"/>
       <c r="G11" s="3"/>
@@ -5410,7 +5410,7 @@
       <c r="K11" s="3"/>
       <c r="L11" s="3"/>
       <c r="M11" s="8" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="N11" s="3" t="s">
         <v>5</v>
@@ -5430,7 +5430,7 @@
         <v>84</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="F12" s="3"/>
       <c r="G12" s="3"/>
@@ -5440,7 +5440,7 @@
       <c r="K12" s="3"/>
       <c r="L12" s="3"/>
       <c r="M12" s="8" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="N12" s="3" t="s">
         <v>5</v>
@@ -5457,10 +5457,10 @@
         <v>138</v>
       </c>
       <c r="D13" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="E13" s="3" t="s">
         <v>216</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>217</v>
       </c>
       <c r="F13" s="3"/>
       <c r="G13" s="3"/>
@@ -5470,7 +5470,7 @@
       <c r="K13" s="3"/>
       <c r="L13" s="3"/>
       <c r="M13" s="8" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="N13" s="3" t="s">
         <v>5</v>
@@ -5490,7 +5490,7 @@
         <v>85</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="F14" s="3"/>
       <c r="G14" s="3"/>
@@ -5500,7 +5500,7 @@
       <c r="K14" s="3"/>
       <c r="L14" s="3"/>
       <c r="M14" s="8" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="N14" s="3" t="s">
         <v>5</v>
@@ -5520,10 +5520,10 @@
         <v>86</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="G15" s="3"/>
       <c r="H15" s="3"/>
@@ -5532,7 +5532,7 @@
       <c r="K15" s="3"/>
       <c r="L15" s="3"/>
       <c r="M15" s="3" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="N15" s="3" t="s">
         <v>5</v>
@@ -5552,7 +5552,7 @@
         <v>87</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="F16" s="3"/>
       <c r="G16" s="3"/>
@@ -5562,7 +5562,7 @@
       <c r="K16" s="3"/>
       <c r="L16" s="3"/>
       <c r="M16" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="N16" s="3" t="s">
         <v>5</v>
@@ -5582,10 +5582,10 @@
         <v>88</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="G17" s="3"/>
       <c r="H17" s="3"/>
@@ -5614,7 +5614,7 @@
         <v>89</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="F18" s="3"/>
       <c r="G18" s="3"/>
@@ -5624,7 +5624,7 @@
       <c r="K18" s="3"/>
       <c r="L18" s="3"/>
       <c r="M18" s="3" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="N18" s="3" t="s">
         <v>5</v>
@@ -5644,7 +5644,7 @@
         <v>90</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="F19" s="3"/>
       <c r="G19" s="3"/>
@@ -5654,7 +5654,7 @@
       <c r="K19" s="3"/>
       <c r="L19" s="3"/>
       <c r="M19" s="3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="N19" s="3" t="s">
         <v>5</v>
@@ -5674,7 +5674,7 @@
         <v>91</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="F20" s="3"/>
       <c r="G20" s="3"/>
@@ -5684,7 +5684,7 @@
       <c r="K20" s="3"/>
       <c r="L20" s="3"/>
       <c r="M20" s="3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="N20" s="3" t="s">
         <v>5</v>
@@ -5704,7 +5704,7 @@
         <v>92</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="F21" s="3"/>
       <c r="G21" s="3"/>
@@ -5714,7 +5714,7 @@
       <c r="K21" s="3"/>
       <c r="L21" s="3"/>
       <c r="M21" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="N21" s="3" t="s">
         <v>5</v>
@@ -5734,7 +5734,7 @@
         <v>93</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="F22" s="3"/>
       <c r="G22" s="3"/>
@@ -5764,7 +5764,7 @@
         <v>94</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="F23" s="3"/>
       <c r="G23" s="3"/>
@@ -5774,7 +5774,7 @@
       <c r="K23" s="3"/>
       <c r="L23" s="3"/>
       <c r="M23" s="8" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="N23" s="3" t="s">
         <v>5</v>
@@ -5794,7 +5794,7 @@
         <v>95</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="F24" s="3"/>
       <c r="G24" s="3"/>
@@ -5804,7 +5804,7 @@
       <c r="K24" s="3"/>
       <c r="L24" s="3"/>
       <c r="M24" s="8" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="N24" s="3" t="s">
         <v>5</v>
@@ -5818,13 +5818,13 @@
         <v>11</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="D25" s="3" t="s">
         <v>96</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="F25" s="3"/>
       <c r="G25" s="3"/>
@@ -5834,7 +5834,7 @@
       <c r="K25" s="3"/>
       <c r="L25" s="3"/>
       <c r="M25" s="8" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="N25" s="3" t="s">
         <v>5</v>
@@ -5854,7 +5854,7 @@
         <v>97</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="F26" s="3"/>
       <c r="G26" s="3"/>
@@ -5864,7 +5864,7 @@
       <c r="K26" s="3"/>
       <c r="L26" s="3"/>
       <c r="M26" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="N26" s="3" t="s">
         <v>5</v>
@@ -5884,7 +5884,7 @@
         <v>98</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="F27" s="3"/>
       <c r="G27" s="3"/>
@@ -5914,7 +5914,7 @@
         <v>99</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="F28" s="3"/>
       <c r="G28" s="3"/>
@@ -5924,7 +5924,7 @@
       <c r="K28" s="3"/>
       <c r="L28" s="3"/>
       <c r="M28" s="8" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="N28" s="3" t="s">
         <v>5</v>
@@ -5944,7 +5944,7 @@
         <v>100</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="F29" s="3"/>
       <c r="G29" s="3"/>
@@ -5954,7 +5954,7 @@
       <c r="K29" s="3"/>
       <c r="L29" s="3"/>
       <c r="M29" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="N29" s="3" t="s">
         <v>5</v>
@@ -5974,10 +5974,10 @@
         <v>101</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="G30" s="3"/>
       <c r="H30" s="3"/>
@@ -6006,7 +6006,7 @@
         <v>102</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="F31" s="3"/>
       <c r="G31" s="3"/>
@@ -6016,7 +6016,7 @@
       <c r="K31" s="3"/>
       <c r="L31" s="3"/>
       <c r="M31" s="4" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="N31" s="3" t="s">
         <v>5</v>
@@ -6033,10 +6033,10 @@
         <v>156</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="F32" s="3"/>
       <c r="G32" s="3"/>
@@ -6046,7 +6046,7 @@
       <c r="K32" s="3"/>
       <c r="L32" s="3"/>
       <c r="M32" s="3" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="N32" s="3" t="s">
         <v>5</v>
@@ -6063,10 +6063,10 @@
         <v>157</v>
       </c>
       <c r="D33" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="E33" s="3" t="s">
         <v>244</v>
-      </c>
-      <c r="E33" s="3" t="s">
-        <v>245</v>
       </c>
       <c r="F33" s="3"/>
       <c r="G33" s="3"/>
@@ -6096,7 +6096,7 @@
         <v>103</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="F34" s="3"/>
       <c r="G34" s="3"/>
@@ -6120,13 +6120,13 @@
         <v>11</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="F35" s="3"/>
       <c r="G35" s="3"/>
@@ -6136,7 +6136,7 @@
       <c r="K35" s="3"/>
       <c r="L35" s="3"/>
       <c r="M35" s="8" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="N35" s="3" t="s">
         <v>5</v>
@@ -6153,10 +6153,10 @@
         <v>159</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F36" s="3"/>
       <c r="G36" s="3"/>
@@ -6166,7 +6166,7 @@
       <c r="K36" s="3"/>
       <c r="L36" s="3"/>
       <c r="M36" s="8" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="N36" s="3" t="s">
         <v>5</v>
@@ -6183,10 +6183,10 @@
         <v>160</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="F37" s="3"/>
       <c r="G37" s="3"/>
@@ -6196,7 +6196,7 @@
       <c r="K37" s="3"/>
       <c r="L37" s="3"/>
       <c r="M37" s="8" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="N37" s="3" t="s">
         <v>5</v>
@@ -6216,7 +6216,7 @@
         <v>104</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="F38" s="3"/>
       <c r="G38" s="3"/>
@@ -6226,7 +6226,7 @@
       <c r="K38" s="3"/>
       <c r="L38" s="3"/>
       <c r="M38" s="8" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="N38" s="3" t="s">
         <v>5</v>
@@ -6246,7 +6246,7 @@
         <v>105</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="F39" s="3"/>
       <c r="G39" s="3"/>
@@ -6256,7 +6256,7 @@
       <c r="K39" s="3"/>
       <c r="L39" s="3"/>
       <c r="M39" s="8" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="N39" s="3" t="s">
         <v>5</v>
@@ -6276,7 +6276,7 @@
         <v>106</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="F40" s="3"/>
       <c r="G40" s="3"/>
@@ -6286,7 +6286,7 @@
       <c r="K40" s="3"/>
       <c r="L40" s="3"/>
       <c r="M40" s="8" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="N40" s="3" t="s">
         <v>5</v>
@@ -6306,7 +6306,7 @@
         <v>107</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="F41" s="3"/>
       <c r="G41" s="3"/>
@@ -6316,7 +6316,7 @@
       <c r="K41" s="3"/>
       <c r="L41" s="3"/>
       <c r="M41" s="8" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="N41" s="3" t="s">
         <v>5</v>
@@ -6336,7 +6336,7 @@
         <v>108</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="F42" s="3"/>
       <c r="G42" s="3"/>
@@ -6366,7 +6366,7 @@
         <v>109</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="F43" s="3"/>
       <c r="G43" s="3"/>
@@ -6396,7 +6396,7 @@
         <v>110</v>
       </c>
       <c r="E44" s="3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="F44" s="3"/>
       <c r="G44" s="3"/>
@@ -6406,7 +6406,7 @@
       <c r="K44" s="3"/>
       <c r="L44" s="3"/>
       <c r="M44" s="8" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="N44" s="3" t="s">
         <v>5</v>
@@ -6426,7 +6426,7 @@
         <v>111</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="F45" s="3"/>
       <c r="G45" s="3"/>
@@ -6436,7 +6436,7 @@
       <c r="K45" s="3"/>
       <c r="L45" s="3"/>
       <c r="M45" s="8" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="N45" s="3" t="s">
         <v>5</v>
@@ -6456,21 +6456,21 @@
         <v>112</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F46" s="3" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="G46" s="3"/>
       <c r="H46" s="9" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="I46" s="3"/>
       <c r="J46" s="3"/>
       <c r="K46" s="3"/>
       <c r="L46" s="3"/>
       <c r="M46" s="3" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="N46" s="3" t="s">
         <v>5</v>
@@ -6490,7 +6490,7 @@
         <v>113</v>
       </c>
       <c r="E47" s="3" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F47" s="3"/>
       <c r="G47" s="3"/>
@@ -6500,7 +6500,7 @@
       <c r="K47" s="3"/>
       <c r="L47" s="3"/>
       <c r="M47" s="3" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="N47" s="3" t="s">
         <v>5</v>
@@ -6520,7 +6520,7 @@
         <v>114</v>
       </c>
       <c r="E48" s="3" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="F48" s="3"/>
       <c r="G48" s="3"/>
@@ -6530,7 +6530,7 @@
       <c r="K48" s="3"/>
       <c r="L48" s="3"/>
       <c r="M48" s="8" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="N48" s="3" t="s">
         <v>5</v>
@@ -6550,7 +6550,7 @@
         <v>115</v>
       </c>
       <c r="E49" s="3" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="F49" s="3"/>
       <c r="G49" s="3"/>
@@ -6560,7 +6560,7 @@
       <c r="K49" s="3"/>
       <c r="L49" s="3"/>
       <c r="M49" s="8" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="N49" s="3" t="s">
         <v>5</v>
@@ -6580,7 +6580,7 @@
         <v>116</v>
       </c>
       <c r="E50" s="3" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="F50" s="3"/>
       <c r="G50" s="3"/>
@@ -6610,7 +6610,7 @@
         <v>117</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="F51" s="3"/>
       <c r="G51" s="3"/>
@@ -6620,7 +6620,7 @@
       <c r="K51" s="3"/>
       <c r="L51" s="3"/>
       <c r="M51" s="3" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="N51" s="3" t="s">
         <v>5</v>
@@ -6640,21 +6640,21 @@
         <v>118</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F52" s="3" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="G52" s="3"/>
       <c r="H52" s="9" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="I52" s="3"/>
       <c r="J52" s="3"/>
       <c r="K52" s="3"/>
       <c r="L52" s="3"/>
       <c r="M52" s="8" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="N52" s="3" t="s">
         <v>5</v>
@@ -6674,7 +6674,7 @@
         <v>119</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="F53" s="3"/>
       <c r="G53" s="3"/>
@@ -6684,7 +6684,7 @@
       <c r="K53" s="3"/>
       <c r="L53" s="3"/>
       <c r="M53" s="3" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="N53" s="3" t="s">
         <v>5</v>
@@ -6704,7 +6704,7 @@
         <v>120</v>
       </c>
       <c r="E54" s="3" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="F54" s="3"/>
       <c r="G54" s="3"/>
@@ -6714,7 +6714,7 @@
       <c r="K54" s="3"/>
       <c r="L54" s="3"/>
       <c r="M54" s="8" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="N54" s="3" t="s">
         <v>5</v>
@@ -6734,7 +6734,7 @@
         <v>121</v>
       </c>
       <c r="E55" s="3" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="F55" s="3"/>
       <c r="G55" s="3"/>
@@ -6764,7 +6764,7 @@
         <v>122</v>
       </c>
       <c r="E56" s="3" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="F56" s="3"/>
       <c r="G56" s="3"/>
@@ -6774,7 +6774,7 @@
       <c r="K56" s="3"/>
       <c r="L56" s="3"/>
       <c r="M56" s="8" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="N56" s="3" t="s">
         <v>5</v>
@@ -6794,7 +6794,7 @@
         <v>123</v>
       </c>
       <c r="E57" s="3" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="F57" s="3"/>
       <c r="G57" s="3"/>
@@ -6804,7 +6804,7 @@
       <c r="K57" s="3"/>
       <c r="L57" s="3"/>
       <c r="M57" s="8" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="N57" s="3" t="s">
         <v>5</v>
@@ -7136,7 +7136,7 @@
         <v>22</v>
       </c>
       <c r="E68" s="3" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="F68" s="3"/>
       <c r="G68" s="3"/>
@@ -7172,7 +7172,7 @@
         <v>124</v>
       </c>
       <c r="E69" s="3" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="F69" s="3"/>
       <c r="G69" s="3"/>
@@ -7182,7 +7182,7 @@
       <c r="K69" s="3"/>
       <c r="L69" s="3"/>
       <c r="M69" s="8" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="N69" s="3" t="s">
         <v>5</v>
@@ -7202,7 +7202,7 @@
         <v>125</v>
       </c>
       <c r="E70" s="3" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="F70" s="3"/>
       <c r="G70" s="3"/>
@@ -7230,7 +7230,7 @@
         <v>126</v>
       </c>
       <c r="E71" s="3" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="F71" s="3"/>
       <c r="G71" s="3"/>
@@ -7240,7 +7240,7 @@
       <c r="K71" s="3"/>
       <c r="L71" s="3"/>
       <c r="M71" s="6" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="N71" s="3" t="s">
         <v>5</v>
@@ -7300,7 +7300,7 @@
       <c r="K73" s="3"/>
       <c r="L73" s="3"/>
       <c r="M73" s="6" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="N73" s="3" t="s">
         <v>5</v>
@@ -7440,7 +7440,7 @@
         <v>29</v>
       </c>
       <c r="E78" s="3" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F78" s="3"/>
       <c r="G78" s="3"/>
@@ -7470,7 +7470,7 @@
         <v>127</v>
       </c>
       <c r="E79" s="3" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="F79" s="3"/>
       <c r="G79" s="3"/>
@@ -7480,7 +7480,7 @@
       <c r="K79" s="3"/>
       <c r="L79" s="3"/>
       <c r="M79" s="6" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="N79" s="3" t="s">
         <v>5</v>

</xml_diff>

<commit_message>
Resolved Failed Test cases - 12-Jun-2026
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/Modules/09_MyWebSite/MyWebSite/02_WebSite_Resubmit.xlsx
+++ b/src/test/resources/testdata/Modules/09_MyWebSite/MyWebSite/02_WebSite_Resubmit.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\testing\Documents\Bandhan_World_APPIUM\src\test\resources\testdata\Modules\09_MyWebSite\MyWebSite\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{022BA03F-DDCC-4736-95E6-4ED350673D5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CFE10EC-6C9C-4A12-8B79-1667F5377A19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="1" xr2:uid="{D5674106-8292-4F40-9DFC-E6EAC771FC2F}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{D5674106-8292-4F40-9DFC-E6EAC771FC2F}"/>
   </bookViews>
   <sheets>
     <sheet name="TestCases" sheetId="1" r:id="rId1"/>
@@ -1314,11 +1314,6 @@
     <t>verify_alert_dialog_text</t>
   </si>
   <si>
-    <t>clickon_resubmitdata_clickherebtn
-clickon_alert_dialog_yesbtn
-verify_successdialog_title</t>
-  </si>
-  <si>
     <t>clickon_successdialog_okbtn
 verify_rejectedfieldspage_status_1</t>
   </si>
@@ -1678,6 +1673,12 @@
 clickonskipbtnofinsurancewindow
 open_mywebsitemenu
 verify_resubmit_webvesrion_status</t>
+  </si>
+  <si>
+    <t>clickon_resubmitdata_clickherebtn
+clickon_resubmitdata_clickherebtn
+clickon_alert_dialog_yesbtn
+verify_successdialog_title</t>
   </si>
 </sst>
 </file>
@@ -2717,7 +2718,7 @@
         <v>75</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
@@ -2741,7 +2742,7 @@
         <v>11</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>74</v>
@@ -2817,7 +2818,7 @@
       <c r="K6" s="3"/>
       <c r="L6" s="3"/>
       <c r="M6" s="3" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="N6" s="3" t="s">
         <v>5</v>
@@ -2837,7 +2838,7 @@
         <v>79</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="F7" s="3"/>
       <c r="G7" s="3"/>
@@ -2907,7 +2908,7 @@
       <c r="K9" s="3"/>
       <c r="L9" s="3"/>
       <c r="M9" s="8" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N9" s="3" t="s">
         <v>5</v>
@@ -3027,7 +3028,7 @@
       <c r="K13" s="3"/>
       <c r="L13" s="3"/>
       <c r="M13" s="8" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="N13" s="3" t="s">
         <v>5</v>
@@ -3077,7 +3078,7 @@
         <v>86</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="F15" s="3" t="s">
         <v>221</v>
@@ -3351,7 +3352,7 @@
         <v>95</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="F24" s="3"/>
       <c r="G24" s="3"/>
@@ -3375,7 +3376,7 @@
         <v>11</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="D25" s="3" t="s">
         <v>96</v>
@@ -3391,7 +3392,7 @@
       <c r="K25" s="3"/>
       <c r="L25" s="3"/>
       <c r="M25" s="8" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="N25" s="3" t="s">
         <v>5</v>
@@ -3411,7 +3412,7 @@
         <v>97</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="F26" s="3"/>
       <c r="G26" s="3"/>
@@ -3427,7 +3428,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="27" spans="1:14" s="5" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:14" s="5" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A27" s="3" t="s">
         <v>8</v>
       </c>
@@ -3441,7 +3442,7 @@
         <v>98</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>234</v>
+        <v>311</v>
       </c>
       <c r="F27" s="3"/>
       <c r="G27" s="3"/>
@@ -3471,7 +3472,7 @@
         <v>99</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="F28" s="3"/>
       <c r="G28" s="3"/>
@@ -3481,7 +3482,7 @@
       <c r="K28" s="3"/>
       <c r="L28" s="3"/>
       <c r="M28" s="8" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="N28" s="3" t="s">
         <v>5</v>
@@ -3501,7 +3502,7 @@
         <v>100</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="F29" s="3"/>
       <c r="G29" s="3"/>
@@ -3531,10 +3532,10 @@
         <v>101</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="G30" s="3"/>
       <c r="H30" s="3"/>
@@ -3563,7 +3564,7 @@
         <v>102</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="F31" s="3"/>
       <c r="G31" s="3"/>
@@ -3590,10 +3591,10 @@
         <v>156</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="F32" s="3"/>
       <c r="G32" s="3"/>
@@ -3603,7 +3604,7 @@
       <c r="K32" s="3"/>
       <c r="L32" s="3"/>
       <c r="M32" s="3" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="N32" s="3" t="s">
         <v>5</v>
@@ -3620,10 +3621,10 @@
         <v>157</v>
       </c>
       <c r="D33" s="3" t="s">
+        <v>242</v>
+      </c>
+      <c r="E33" s="3" t="s">
         <v>243</v>
-      </c>
-      <c r="E33" s="3" t="s">
-        <v>244</v>
       </c>
       <c r="F33" s="3"/>
       <c r="G33" s="3"/>
@@ -3653,7 +3654,7 @@
         <v>103</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="F34" s="3"/>
       <c r="G34" s="3"/>
@@ -3677,13 +3678,13 @@
         <v>11</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="F35" s="3"/>
       <c r="G35" s="3"/>
@@ -3693,7 +3694,7 @@
       <c r="K35" s="3"/>
       <c r="L35" s="3"/>
       <c r="M35" s="8" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="N35" s="3" t="s">
         <v>5</v>
@@ -3710,10 +3711,10 @@
         <v>159</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="F36" s="3"/>
       <c r="G36" s="3"/>
@@ -3723,7 +3724,7 @@
       <c r="K36" s="3"/>
       <c r="L36" s="3"/>
       <c r="M36" s="8" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="N36" s="3" t="s">
         <v>5</v>
@@ -3740,10 +3741,10 @@
         <v>160</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F37" s="3"/>
       <c r="G37" s="3"/>
@@ -3753,7 +3754,7 @@
       <c r="K37" s="3"/>
       <c r="L37" s="3"/>
       <c r="M37" s="8" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="N37" s="3" t="s">
         <v>5</v>
@@ -3773,7 +3774,7 @@
         <v>104</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="F38" s="3"/>
       <c r="G38" s="3"/>
@@ -3783,7 +3784,7 @@
       <c r="K38" s="3"/>
       <c r="L38" s="3"/>
       <c r="M38" s="8" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="N38" s="3" t="s">
         <v>5</v>
@@ -3803,7 +3804,7 @@
         <v>105</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="F39" s="3"/>
       <c r="G39" s="3"/>
@@ -3813,7 +3814,7 @@
       <c r="K39" s="3"/>
       <c r="L39" s="3"/>
       <c r="M39" s="8" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="N39" s="3" t="s">
         <v>5</v>
@@ -3833,7 +3834,7 @@
         <v>106</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="F40" s="3"/>
       <c r="G40" s="3"/>
@@ -3843,7 +3844,7 @@
       <c r="K40" s="3"/>
       <c r="L40" s="3"/>
       <c r="M40" s="8" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="N40" s="3" t="s">
         <v>5</v>
@@ -3863,7 +3864,7 @@
         <v>107</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="F41" s="3"/>
       <c r="G41" s="3"/>
@@ -3873,7 +3874,7 @@
       <c r="K41" s="3"/>
       <c r="L41" s="3"/>
       <c r="M41" s="8" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="N41" s="3" t="s">
         <v>5</v>
@@ -3893,7 +3894,7 @@
         <v>108</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="F42" s="3"/>
       <c r="G42" s="3"/>
@@ -3923,7 +3924,7 @@
         <v>109</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="F43" s="3"/>
       <c r="G43" s="3"/>
@@ -3953,7 +3954,7 @@
         <v>110</v>
       </c>
       <c r="E44" s="3" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="F44" s="3"/>
       <c r="G44" s="3"/>
@@ -3963,7 +3964,7 @@
       <c r="K44" s="3"/>
       <c r="L44" s="3"/>
       <c r="M44" s="8" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="N44" s="3" t="s">
         <v>5</v>
@@ -3983,7 +3984,7 @@
         <v>111</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="F45" s="3"/>
       <c r="G45" s="3"/>
@@ -3993,7 +3994,7 @@
       <c r="K45" s="3"/>
       <c r="L45" s="3"/>
       <c r="M45" s="8" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="N45" s="3" t="s">
         <v>5</v>
@@ -4013,21 +4014,21 @@
         <v>112</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F46" s="3" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="G46" s="3"/>
       <c r="H46" s="9" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="I46" s="3"/>
       <c r="J46" s="3"/>
       <c r="K46" s="3"/>
       <c r="L46" s="3"/>
       <c r="M46" s="3" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="N46" s="3" t="s">
         <v>5</v>
@@ -4047,7 +4048,7 @@
         <v>113</v>
       </c>
       <c r="E47" s="3" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F47" s="3"/>
       <c r="G47" s="3"/>
@@ -4057,7 +4058,7 @@
       <c r="K47" s="3"/>
       <c r="L47" s="3"/>
       <c r="M47" s="3" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="N47" s="3" t="s">
         <v>5</v>
@@ -4077,7 +4078,7 @@
         <v>114</v>
       </c>
       <c r="E48" s="3" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="F48" s="3"/>
       <c r="G48" s="3"/>
@@ -4087,7 +4088,7 @@
       <c r="K48" s="3"/>
       <c r="L48" s="3"/>
       <c r="M48" s="8" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="N48" s="3" t="s">
         <v>5</v>
@@ -4107,7 +4108,7 @@
         <v>115</v>
       </c>
       <c r="E49" s="3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="F49" s="3"/>
       <c r="G49" s="3"/>
@@ -4117,7 +4118,7 @@
       <c r="K49" s="3"/>
       <c r="L49" s="3"/>
       <c r="M49" s="8" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="N49" s="3" t="s">
         <v>5</v>
@@ -4137,7 +4138,7 @@
         <v>116</v>
       </c>
       <c r="E50" s="3" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="F50" s="3"/>
       <c r="G50" s="3"/>
@@ -4167,7 +4168,7 @@
         <v>117</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="F51" s="3"/>
       <c r="G51" s="3"/>
@@ -4177,7 +4178,7 @@
       <c r="K51" s="3"/>
       <c r="L51" s="3"/>
       <c r="M51" s="3" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="N51" s="3" t="s">
         <v>5</v>
@@ -4197,21 +4198,21 @@
         <v>118</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="F52" s="3" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="G52" s="3"/>
       <c r="H52" s="9" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="I52" s="3"/>
       <c r="J52" s="3"/>
       <c r="K52" s="3"/>
       <c r="L52" s="3"/>
       <c r="M52" s="8" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="N52" s="3" t="s">
         <v>5</v>
@@ -4231,7 +4232,7 @@
         <v>119</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F53" s="3"/>
       <c r="G53" s="3"/>
@@ -4241,7 +4242,7 @@
       <c r="K53" s="3"/>
       <c r="L53" s="3"/>
       <c r="M53" s="3" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="N53" s="3" t="s">
         <v>5</v>
@@ -4261,7 +4262,7 @@
         <v>120</v>
       </c>
       <c r="E54" s="3" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="F54" s="3"/>
       <c r="G54" s="3"/>
@@ -4271,7 +4272,7 @@
       <c r="K54" s="3"/>
       <c r="L54" s="3"/>
       <c r="M54" s="8" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="N54" s="3" t="s">
         <v>5</v>
@@ -4291,7 +4292,7 @@
         <v>121</v>
       </c>
       <c r="E55" s="3" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="F55" s="3"/>
       <c r="G55" s="3"/>
@@ -4321,7 +4322,7 @@
         <v>122</v>
       </c>
       <c r="E56" s="3" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="F56" s="3"/>
       <c r="G56" s="3"/>
@@ -4331,7 +4332,7 @@
       <c r="K56" s="3"/>
       <c r="L56" s="3"/>
       <c r="M56" s="8" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="N56" s="3" t="s">
         <v>5</v>
@@ -4351,7 +4352,7 @@
         <v>123</v>
       </c>
       <c r="E57" s="3" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="F57" s="3"/>
       <c r="G57" s="3"/>
@@ -4361,7 +4362,7 @@
       <c r="K57" s="3"/>
       <c r="L57" s="3"/>
       <c r="M57" s="8" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="N57" s="3" t="s">
         <v>5</v>
@@ -4693,7 +4694,7 @@
         <v>22</v>
       </c>
       <c r="E68" s="3" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="F68" s="3"/>
       <c r="G68" s="3"/>
@@ -4729,7 +4730,7 @@
         <v>124</v>
       </c>
       <c r="E69" s="3" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="F69" s="3"/>
       <c r="G69" s="3"/>
@@ -4739,7 +4740,7 @@
       <c r="K69" s="3"/>
       <c r="L69" s="3"/>
       <c r="M69" s="8" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="N69" s="3" t="s">
         <v>5</v>
@@ -4759,7 +4760,7 @@
         <v>125</v>
       </c>
       <c r="E70" s="3" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="F70" s="3"/>
       <c r="G70" s="3"/>
@@ -4787,7 +4788,7 @@
         <v>126</v>
       </c>
       <c r="E71" s="3" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="F71" s="3"/>
       <c r="G71" s="3"/>
@@ -4797,7 +4798,7 @@
       <c r="K71" s="3"/>
       <c r="L71" s="3"/>
       <c r="M71" s="6" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="N71" s="3" t="s">
         <v>5</v>
@@ -4857,7 +4858,7 @@
       <c r="K73" s="3"/>
       <c r="L73" s="3"/>
       <c r="M73" s="6" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="N73" s="3" t="s">
         <v>5</v>
@@ -4997,7 +4998,7 @@
         <v>29</v>
       </c>
       <c r="E78" s="3" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="F78" s="3"/>
       <c r="G78" s="3"/>
@@ -5027,7 +5028,7 @@
         <v>127</v>
       </c>
       <c r="E79" s="3" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F79" s="3"/>
       <c r="G79" s="3"/>
@@ -5037,7 +5038,7 @@
       <c r="K79" s="3"/>
       <c r="L79" s="3"/>
       <c r="M79" s="6" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="N79" s="3" t="s">
         <v>5</v>
@@ -5160,7 +5161,7 @@
         <v>75</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
@@ -5184,7 +5185,7 @@
         <v>11</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>74</v>
@@ -5260,7 +5261,7 @@
       <c r="K6" s="3"/>
       <c r="L6" s="3"/>
       <c r="M6" s="3" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="N6" s="3" t="s">
         <v>5</v>
@@ -5280,7 +5281,7 @@
         <v>79</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="F7" s="3"/>
       <c r="G7" s="3"/>
@@ -5350,7 +5351,7 @@
       <c r="K9" s="3"/>
       <c r="L9" s="3"/>
       <c r="M9" s="8" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="N9" s="3" t="s">
         <v>5</v>
@@ -5470,7 +5471,7 @@
       <c r="K13" s="3"/>
       <c r="L13" s="3"/>
       <c r="M13" s="8" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="N13" s="3" t="s">
         <v>5</v>
@@ -5520,7 +5521,7 @@
         <v>86</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="F15" s="3" t="s">
         <v>221</v>
@@ -5794,7 +5795,7 @@
         <v>95</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="F24" s="3"/>
       <c r="G24" s="3"/>
@@ -5818,7 +5819,7 @@
         <v>11</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="D25" s="3" t="s">
         <v>96</v>
@@ -5834,7 +5835,7 @@
       <c r="K25" s="3"/>
       <c r="L25" s="3"/>
       <c r="M25" s="8" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="N25" s="3" t="s">
         <v>5</v>
@@ -5854,7 +5855,7 @@
         <v>97</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="F26" s="3"/>
       <c r="G26" s="3"/>
@@ -5870,7 +5871,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="27" spans="1:14" s="5" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:14" s="5" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A27" s="3" t="s">
         <v>8</v>
       </c>
@@ -5884,7 +5885,7 @@
         <v>98</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>234</v>
+        <v>311</v>
       </c>
       <c r="F27" s="3"/>
       <c r="G27" s="3"/>
@@ -5914,7 +5915,7 @@
         <v>99</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="F28" s="3"/>
       <c r="G28" s="3"/>
@@ -5924,7 +5925,7 @@
       <c r="K28" s="3"/>
       <c r="L28" s="3"/>
       <c r="M28" s="8" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="N28" s="3" t="s">
         <v>5</v>
@@ -5944,7 +5945,7 @@
         <v>100</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="F29" s="3"/>
       <c r="G29" s="3"/>
@@ -5974,10 +5975,10 @@
         <v>101</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="G30" s="3"/>
       <c r="H30" s="3"/>
@@ -6006,7 +6007,7 @@
         <v>102</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="F31" s="3"/>
       <c r="G31" s="3"/>
@@ -6033,10 +6034,10 @@
         <v>156</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="F32" s="3"/>
       <c r="G32" s="3"/>
@@ -6046,7 +6047,7 @@
       <c r="K32" s="3"/>
       <c r="L32" s="3"/>
       <c r="M32" s="3" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="N32" s="3" t="s">
         <v>5</v>
@@ -6063,10 +6064,10 @@
         <v>157</v>
       </c>
       <c r="D33" s="3" t="s">
+        <v>242</v>
+      </c>
+      <c r="E33" s="3" t="s">
         <v>243</v>
-      </c>
-      <c r="E33" s="3" t="s">
-        <v>244</v>
       </c>
       <c r="F33" s="3"/>
       <c r="G33" s="3"/>
@@ -6096,7 +6097,7 @@
         <v>103</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="F34" s="3"/>
       <c r="G34" s="3"/>
@@ -6120,13 +6121,13 @@
         <v>11</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="F35" s="3"/>
       <c r="G35" s="3"/>
@@ -6136,7 +6137,7 @@
       <c r="K35" s="3"/>
       <c r="L35" s="3"/>
       <c r="M35" s="8" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="N35" s="3" t="s">
         <v>5</v>
@@ -6153,10 +6154,10 @@
         <v>159</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="F36" s="3"/>
       <c r="G36" s="3"/>
@@ -6166,7 +6167,7 @@
       <c r="K36" s="3"/>
       <c r="L36" s="3"/>
       <c r="M36" s="8" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="N36" s="3" t="s">
         <v>5</v>
@@ -6183,10 +6184,10 @@
         <v>160</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F37" s="3"/>
       <c r="G37" s="3"/>
@@ -6196,7 +6197,7 @@
       <c r="K37" s="3"/>
       <c r="L37" s="3"/>
       <c r="M37" s="8" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="N37" s="3" t="s">
         <v>5</v>
@@ -6216,7 +6217,7 @@
         <v>104</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="F38" s="3"/>
       <c r="G38" s="3"/>
@@ -6226,7 +6227,7 @@
       <c r="K38" s="3"/>
       <c r="L38" s="3"/>
       <c r="M38" s="8" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="N38" s="3" t="s">
         <v>5</v>
@@ -6246,7 +6247,7 @@
         <v>105</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="F39" s="3"/>
       <c r="G39" s="3"/>
@@ -6256,7 +6257,7 @@
       <c r="K39" s="3"/>
       <c r="L39" s="3"/>
       <c r="M39" s="8" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="N39" s="3" t="s">
         <v>5</v>
@@ -6276,7 +6277,7 @@
         <v>106</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="F40" s="3"/>
       <c r="G40" s="3"/>
@@ -6286,7 +6287,7 @@
       <c r="K40" s="3"/>
       <c r="L40" s="3"/>
       <c r="M40" s="8" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="N40" s="3" t="s">
         <v>5</v>
@@ -6306,7 +6307,7 @@
         <v>107</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="F41" s="3"/>
       <c r="G41" s="3"/>
@@ -6316,7 +6317,7 @@
       <c r="K41" s="3"/>
       <c r="L41" s="3"/>
       <c r="M41" s="8" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="N41" s="3" t="s">
         <v>5</v>
@@ -6336,7 +6337,7 @@
         <v>108</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="F42" s="3"/>
       <c r="G42" s="3"/>
@@ -6366,7 +6367,7 @@
         <v>109</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="F43" s="3"/>
       <c r="G43" s="3"/>
@@ -6396,7 +6397,7 @@
         <v>110</v>
       </c>
       <c r="E44" s="3" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="F44" s="3"/>
       <c r="G44" s="3"/>
@@ -6406,7 +6407,7 @@
       <c r="K44" s="3"/>
       <c r="L44" s="3"/>
       <c r="M44" s="8" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="N44" s="3" t="s">
         <v>5</v>
@@ -6426,7 +6427,7 @@
         <v>111</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="F45" s="3"/>
       <c r="G45" s="3"/>
@@ -6436,7 +6437,7 @@
       <c r="K45" s="3"/>
       <c r="L45" s="3"/>
       <c r="M45" s="8" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="N45" s="3" t="s">
         <v>5</v>
@@ -6456,21 +6457,21 @@
         <v>112</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F46" s="3" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="G46" s="3"/>
       <c r="H46" s="9" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="I46" s="3"/>
       <c r="J46" s="3"/>
       <c r="K46" s="3"/>
       <c r="L46" s="3"/>
       <c r="M46" s="3" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="N46" s="3" t="s">
         <v>5</v>
@@ -6490,7 +6491,7 @@
         <v>113</v>
       </c>
       <c r="E47" s="3" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F47" s="3"/>
       <c r="G47" s="3"/>
@@ -6500,7 +6501,7 @@
       <c r="K47" s="3"/>
       <c r="L47" s="3"/>
       <c r="M47" s="3" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="N47" s="3" t="s">
         <v>5</v>
@@ -6520,7 +6521,7 @@
         <v>114</v>
       </c>
       <c r="E48" s="3" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="F48" s="3"/>
       <c r="G48" s="3"/>
@@ -6530,7 +6531,7 @@
       <c r="K48" s="3"/>
       <c r="L48" s="3"/>
       <c r="M48" s="8" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="N48" s="3" t="s">
         <v>5</v>
@@ -6550,7 +6551,7 @@
         <v>115</v>
       </c>
       <c r="E49" s="3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="F49" s="3"/>
       <c r="G49" s="3"/>
@@ -6560,7 +6561,7 @@
       <c r="K49" s="3"/>
       <c r="L49" s="3"/>
       <c r="M49" s="8" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="N49" s="3" t="s">
         <v>5</v>
@@ -6580,7 +6581,7 @@
         <v>116</v>
       </c>
       <c r="E50" s="3" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="F50" s="3"/>
       <c r="G50" s="3"/>
@@ -6610,7 +6611,7 @@
         <v>117</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="F51" s="3"/>
       <c r="G51" s="3"/>
@@ -6620,7 +6621,7 @@
       <c r="K51" s="3"/>
       <c r="L51" s="3"/>
       <c r="M51" s="3" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="N51" s="3" t="s">
         <v>5</v>
@@ -6640,21 +6641,21 @@
         <v>118</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="F52" s="3" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="G52" s="3"/>
       <c r="H52" s="9" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="I52" s="3"/>
       <c r="J52" s="3"/>
       <c r="K52" s="3"/>
       <c r="L52" s="3"/>
       <c r="M52" s="8" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="N52" s="3" t="s">
         <v>5</v>
@@ -6674,7 +6675,7 @@
         <v>119</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F53" s="3"/>
       <c r="G53" s="3"/>
@@ -6684,7 +6685,7 @@
       <c r="K53" s="3"/>
       <c r="L53" s="3"/>
       <c r="M53" s="3" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="N53" s="3" t="s">
         <v>5</v>
@@ -6704,7 +6705,7 @@
         <v>120</v>
       </c>
       <c r="E54" s="3" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="F54" s="3"/>
       <c r="G54" s="3"/>
@@ -6714,7 +6715,7 @@
       <c r="K54" s="3"/>
       <c r="L54" s="3"/>
       <c r="M54" s="8" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="N54" s="3" t="s">
         <v>5</v>
@@ -6734,7 +6735,7 @@
         <v>121</v>
       </c>
       <c r="E55" s="3" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="F55" s="3"/>
       <c r="G55" s="3"/>
@@ -6764,7 +6765,7 @@
         <v>122</v>
       </c>
       <c r="E56" s="3" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="F56" s="3"/>
       <c r="G56" s="3"/>
@@ -6774,7 +6775,7 @@
       <c r="K56" s="3"/>
       <c r="L56" s="3"/>
       <c r="M56" s="8" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="N56" s="3" t="s">
         <v>5</v>
@@ -6794,7 +6795,7 @@
         <v>123</v>
       </c>
       <c r="E57" s="3" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="F57" s="3"/>
       <c r="G57" s="3"/>
@@ -6804,7 +6805,7 @@
       <c r="K57" s="3"/>
       <c r="L57" s="3"/>
       <c r="M57" s="8" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="N57" s="3" t="s">
         <v>5</v>
@@ -7136,7 +7137,7 @@
         <v>22</v>
       </c>
       <c r="E68" s="3" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="F68" s="3"/>
       <c r="G68" s="3"/>
@@ -7172,7 +7173,7 @@
         <v>124</v>
       </c>
       <c r="E69" s="3" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="F69" s="3"/>
       <c r="G69" s="3"/>
@@ -7182,7 +7183,7 @@
       <c r="K69" s="3"/>
       <c r="L69" s="3"/>
       <c r="M69" s="8" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="N69" s="3" t="s">
         <v>5</v>
@@ -7202,7 +7203,7 @@
         <v>125</v>
       </c>
       <c r="E70" s="3" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="F70" s="3"/>
       <c r="G70" s="3"/>
@@ -7230,7 +7231,7 @@
         <v>126</v>
       </c>
       <c r="E71" s="3" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="F71" s="3"/>
       <c r="G71" s="3"/>
@@ -7240,7 +7241,7 @@
       <c r="K71" s="3"/>
       <c r="L71" s="3"/>
       <c r="M71" s="6" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="N71" s="3" t="s">
         <v>5</v>
@@ -7300,7 +7301,7 @@
       <c r="K73" s="3"/>
       <c r="L73" s="3"/>
       <c r="M73" s="6" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="N73" s="3" t="s">
         <v>5</v>
@@ -7440,7 +7441,7 @@
         <v>29</v>
       </c>
       <c r="E78" s="3" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="F78" s="3"/>
       <c r="G78" s="3"/>
@@ -7470,7 +7471,7 @@
         <v>127</v>
       </c>
       <c r="E79" s="3" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F79" s="3"/>
       <c r="G79" s="3"/>
@@ -7480,7 +7481,7 @@
       <c r="K79" s="3"/>
       <c r="L79" s="3"/>
       <c r="M79" s="6" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="N79" s="3" t="s">
         <v>5</v>

</xml_diff>

<commit_message>
MyWebSite Module TestCases updated
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/Modules/09_MyWebSite/MyWebSite/02_WebSite_Resubmit.xlsx
+++ b/src/test/resources/testdata/Modules/09_MyWebSite/MyWebSite/02_WebSite_Resubmit.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\testing\Documents\Bandhan_World_APPIUM\src\test\resources\testdata\Modules\09_MyWebSite\MyWebSite\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CFE10EC-6C9C-4A12-8B79-1667F5377A19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E86A229-F2D4-4BD7-8E29-06038A6C0059}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{D5674106-8292-4F40-9DFC-E6EAC771FC2F}"/>
   </bookViews>
   <sheets>
     <sheet name="TestCases" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet1" sheetId="6" r:id="rId2"/>
+    <sheet name="Sheet2" sheetId="7" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="6" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">TestCases!$A$1:$N$1</definedName>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1148" uniqueCount="312">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1169" uniqueCount="312">
   <si>
     <t>TESTCASE_ID</t>
   </si>
@@ -5053,6 +5054,106 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18AB7546-E32C-4130-A639-A02EF63AF89E}">
+  <dimension ref="A1:N2"/>
+  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="12.90625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="13.7265625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="87.81640625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="47" style="1" customWidth="1"/>
+    <col min="6" max="6" width="42.6328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="33.81640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="42.54296875" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21.36328125" style="1" customWidth="1"/>
+    <col min="10" max="11" width="33.36328125" style="1" customWidth="1"/>
+    <col min="12" max="12" width="21.1796875" style="5" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="37.08984375" style="1" customWidth="1"/>
+    <col min="14" max="14" width="10" style="1" customWidth="1"/>
+    <col min="15" max="16384" width="8.90625" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" ht="29" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" s="5" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+      <c r="A2" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3"/>
+      <c r="L2" s="3"/>
+      <c r="M2" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="N2" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0DBF5C95-75F9-4AB2-AC17-2B339FB0566B}">
   <dimension ref="A1:N79"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>

</xml_diff>